<commit_message>
chore(be): add 2 columns in rpg2 statistics
</commit_message>
<xml_diff>
--- a/django/camac/statistics/config/kt_bern/rpg2_service.xlsx
+++ b/django/camac/statistics/config/kt_bern/rpg2_service.xlsx
@@ -740,7 +740,7 @@
         <v>34</v>
       </c>
       <c r="B6">
-        <f>SUM(Flächen!$D:$D)</f>
+        <f>SUBTOTAL(109,Flächen!$D:$D)</f>
         <v>22</v>
       </c>
     </row>
@@ -749,9 +749,7 @@
         <v>35</v>
       </c>
       <c r="B7">
-        <f>SUM(SUMIFS(Dossiers!$J:$J,Dossiers!$M:$M,"Ja",Dossiers!$N:$N,{"Ja",""}))
--SUM(SUMIFS(Dossiers!$K:$K,Dossiers!$M:$M,"Ja",Dossiers!$N:$N,{"Ja",""}))
--SUM(SUMIFS(Dossiers!$L:$L,Dossiers!$M:$M,"Ja",Dossiers!$N:$N,{"Ja",""}))</f>
+        <f>SUBTOTAL(109,Dossiers!$J:$J)-SUBTOTAL(109,Dossiers!$K:$K)-SUBTOTAL(109,Dossiers!$L:$L)</f>
         <v>1</v>
       </c>
     </row>

</xml_diff>